<commit_message>
Styled scoring table; Oakland Campus find folded into Holy Names row; additions.json
- Scoring tab (renamed to match Ria's rename): bordered color-coded table (green earners, red safety, blue bonus, grey rules, graded reading bands, violet worked examples)
- data/additions.json: hand-curated updates/new rows merged by build.ts; first entry upgrades Holy Names to on-market with the theoaklandcampus.com Upper Campus Complex link and Elliot's Aug 26 flag
- Sheet replaced in place; map artifact republished

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/exports/biopunk-housing-tracker.xlsx
+++ b/data/exports/biopunk-housing-tracker.xlsx
@@ -5,7 +5,7 @@
   <sheets>
     <sheet name="Start here" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Priority list" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Scoring explained" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Scoring" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Punkhaus" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Femhaus" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Alumhaus" sheetId="6" state="visible" r:id="rId6"/>
@@ -49,7 +49,7 @@
       <color rgb="0092400E"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -91,8 +91,18 @@
         <fgColor rgb="00FEE2E2"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00ECFCCB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EDE9FE"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -105,11 +115,25 @@
         <color rgb="00DDDDDD"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00B7C4BD"/>
+      </left>
+      <right style="thin">
+        <color rgb="00B7C4BD"/>
+      </right>
+      <top style="thin">
+        <color rgb="00B7C4BD"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00B7C4BD"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -162,6 +186,60 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -737,7 +815,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Scoring explained - how the 0-100 number is built, one line per part, with two worked examples.</t>
+          <t>Scoring - how the 0-100 number is built, one line per part, with two worked examples.</t>
         </is>
       </c>
     </row>
@@ -761,7 +839,7 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>SCORING (0-100): distance 35 + price 30 + kitchen 15 + size 20, minus up to 15 for safety (rough blocks and bad reviews), +5 if ready for arrival day. Dead deals score 0; a tourist hotel with no kitchen caps at 40. Full plain-words breakdown on the Scoring explained tab.</t>
+          <t>SCORING (0-100): distance 35 + price 30 + kitchen 15 + size 20, minus up to 15 for safety (rough blocks and bad reviews), +5 if ready for arrival day. Dead deals score 0; a tourist hotel with no kitchen caps at 40. Full plain-words breakdown on the Scoring tab.</t>
         </is>
       </c>
     </row>
@@ -11235,7 +11313,11 @@
           <t>-</t>
         </is>
       </c>
-      <c r="E108" s="17" t="str"/>
+      <c r="E108" s="17" t="inlineStr">
+        <is>
+          <t>The Oakland Campus (BH Properties leasing site)</t>
+        </is>
+      </c>
       <c r="F108" s="17" t="inlineStr">
         <is>
           <t>3500 Mountain Blvd, Oakland hills</t>
@@ -11304,7 +11386,7 @@
       </c>
       <c r="V108" s="17" t="inlineStr">
         <is>
-          <t>dark</t>
+          <t>on-market</t>
         </is>
       </c>
       <c r="W108" s="17" t="inlineStr">
@@ -14415,153 +14497,153 @@
       <c r="C3" s="2" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" s="19" t="inlineStr">
         <is>
           <t>Part</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" s="19" t="inlineStr">
         <is>
           <t>Points</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C4" s="19" t="inlineStr">
         <is>
           <t>In one line</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" s="20" t="inlineStr">
         <is>
           <t>Distance to Frontier Tower</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B5" s="21" t="inlineStr">
         <is>
           <t>up to 35</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C5" s="22" t="inlineStr">
         <is>
           <t>A 10 minute walk gets all 35; points fade to 0 by 45 minutes away.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" s="20" t="inlineStr">
         <is>
           <t>Price per bed</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B6" s="21" t="inlineStr">
         <is>
           <t>up to 30</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C6" s="22" t="inlineStr">
         <is>
           <t>$1,000 a month or less gets all 30; points fade to 0 by $2,200; no price yet gets 5 so it stays visible.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" s="20" t="inlineStr">
         <is>
           <t>Kitchen</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B7" s="21" t="inlineStr">
         <is>
           <t>up to 15</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C7" s="22" t="inlineStr">
         <is>
           <t>Any real kitchen gets 15; no kitchen gets 0; unknown gets 5.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="A8" s="20" t="inlineStr">
         <is>
           <t>Building size</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B8" s="21" t="inlineStr">
         <is>
           <t>up to 20</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C8" s="22" t="inlineStr">
         <is>
           <t>40 to 60 beds is perfect (20); 20 to 39 works as a pair of buildings (12); under 20 gets 4; over 100 gets 12 to 15.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="A9" s="23" t="inlineStr">
         <is>
           <t>Safety</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B9" s="24" t="inlineStr">
         <is>
           <t>up to -15</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C9" s="22" t="inlineStr">
         <is>
           <t>A rough block (Tenderloin, 6th St, Mid-Market) takes off 8, a mixed block takes off 3, and reviews that flag safety take off up to 7 more.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="A10" s="25" t="inlineStr">
         <is>
           <t>Move-in bonus</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B10" s="26" t="inlineStr">
         <is>
           <t>+5</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C10" s="22" t="inlineStr">
         <is>
           <t>A building confirmed ready for arrival day gets 5 extra.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+      <c r="A11" s="27" t="inlineStr">
         <is>
           <t>Dead deal rule</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B11" s="28" t="inlineStr">
         <is>
           <t>score 0</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C11" s="22" t="inlineStr">
         <is>
           <t>Anything taken, sold, or ruled out drops to 0.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="A12" s="27" t="inlineStr">
         <is>
           <t>Hotel rule</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B12" s="28" t="inlineStr">
         <is>
           <t>cap at 40</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C12" s="22" t="inlineStr">
         <is>
           <t>A tourist hotel with no kitchen can never score above 40, however cheap it is.</t>
         </is>
@@ -14573,77 +14655,77 @@
       <c r="C13" s="2" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="A14" s="19" t="inlineStr">
         <is>
           <t>Reading the number</t>
         </is>
       </c>
-      <c r="B14" s="2" t="str"/>
-      <c r="C14" s="2" t="str"/>
+      <c r="B14" s="19" t="str"/>
+      <c r="C14" s="19" t="str"/>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr">
+      <c r="A15" s="20" t="inlineStr">
         <is>
           <t>80 and up</t>
         </is>
       </c>
-      <c r="B15" s="2" t="inlineStr">
+      <c r="B15" s="29" t="inlineStr">
         <is>
           <t>strong fit</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
+      <c r="C15" s="22" t="inlineStr">
         <is>
           <t>Close, affordable, has a kitchen, right size, decent block. Call first.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr">
+      <c r="A16" s="30" t="inlineStr">
         <is>
           <t>60 to 79</t>
         </is>
       </c>
-      <c r="B16" s="2" t="inlineStr">
+      <c r="B16" s="31" t="inlineStr">
         <is>
           <t>good</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr">
+      <c r="C16" s="22" t="inlineStr">
         <is>
           <t>One thing is off, usually price, distance, or the block. Worth a call.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+      <c r="A17" s="32" t="inlineStr">
         <is>
           <t>40 to 59</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr">
+      <c r="B17" s="33" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="C17" s="2" t="inlineStr">
+      <c r="C17" s="22" t="inlineStr">
         <is>
           <t>Two things are off, or a cap kicked in. Backups.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="inlineStr">
+      <c r="A18" s="27" t="inlineStr">
         <is>
           <t>under 40</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="B18" s="34" t="inlineStr">
         <is>
           <t>stretch</t>
         </is>
       </c>
-      <c r="C18" s="2" t="inlineStr">
+      <c r="C18" s="22" t="inlineStr">
         <is>
           <t>Far, expensive, no kitchen, or dead. Kept for the record.</t>
         </is>
@@ -14655,26 +14737,26 @@
       <c r="C19" s="2" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="inlineStr">
+      <c r="A20" s="35" t="inlineStr">
         <is>
           <t>Worked example: European Hostel</t>
         </is>
       </c>
-      <c r="B20" s="2" t="str"/>
-      <c r="C20" s="2" t="inlineStr">
+      <c r="B20" s="36" t="str"/>
+      <c r="C20" s="36" t="inlineStr">
         <is>
           <t>Walk 35 + price 30 + kitchen 15 + size 12 = 92. Rough block takes off 8 and bad safety reviews take off 7 (capped at 15 total) = 77. Move-in ready adds 5. Final: 82. Cheap and close, but the reviews are why it is not number 1 anymore.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr">
+      <c r="A21" s="35" t="inlineStr">
         <is>
           <t>Worked example: AAU dorm, 860 Sutter</t>
         </is>
       </c>
-      <c r="B21" s="2" t="str"/>
-      <c r="C21" s="2" t="inlineStr">
+      <c r="B21" s="36" t="str"/>
+      <c r="C21" s="36" t="inlineStr">
         <is>
           <t>Walk 31 + price 30 + kitchen 15 + size 15 = 91. Clean Nob Hill block, nothing comes off. Not confirmed for arrival day, no bonus. Final: 89.</t>
         </is>
@@ -14733,7 +14815,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="56" customHeight="1">
-      <c r="A1" s="19" t="inlineStr">
+      <c r="A1" s="37" t="inlineStr">
         <is>
           <t>Main cohort house, 40 to 50 people, buildings with 35+ beds in SF. This tab is the call sheet AND the log: make the call (Granola on), send Claude the notes, and Last outreach / Latest note / Next check on the row get filled in. Ask for: block of beds from Sept 15, monthly rate per bed, kitchen access, minimum term. Tenant-rights worry: 3-month program, visa-bound residents, everyone vacates at program end.</t>
         </is>
@@ -14857,7 +14939,7 @@
           <t>1</t>
         </is>
       </c>
-      <c r="B3" s="20" t="inlineStr">
+      <c r="B3" s="38" t="inlineStr">
         <is>
           <t>Urbanests</t>
         </is>
@@ -14957,7 +15039,7 @@
           <t>2</t>
         </is>
       </c>
-      <c r="B4" s="20" t="inlineStr">
+      <c r="B4" s="38" t="inlineStr">
         <is>
           <t>Hive Coliving (was Tribe)</t>
         </is>
@@ -15061,7 +15143,7 @@
           <t>3</t>
         </is>
       </c>
-      <c r="B5" s="20" t="inlineStr">
+      <c r="B5" s="38" t="inlineStr">
         <is>
           <t>UpMarket Residences</t>
         </is>
@@ -15169,7 +15251,7 @@
           <t>4</t>
         </is>
       </c>
-      <c r="B6" s="20" t="inlineStr">
+      <c r="B6" s="38" t="inlineStr">
         <is>
           <t>AAU dorm</t>
         </is>
@@ -15269,7 +15351,7 @@
           <t>5</t>
         </is>
       </c>
-      <c r="B7" s="20" t="inlineStr">
+      <c r="B7" s="38" t="inlineStr">
         <is>
           <t>Brownstone Shared Housing</t>
         </is>
@@ -15373,7 +15455,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="B8" s="20" t="inlineStr">
+      <c r="B8" s="38" t="inlineStr">
         <is>
           <t>AAU dorm</t>
         </is>
@@ -15473,7 +15555,7 @@
           <t>7</t>
         </is>
       </c>
-      <c r="B9" s="20" t="inlineStr">
+      <c r="B9" s="38" t="inlineStr">
         <is>
           <t>AAU dorm</t>
         </is>
@@ -15573,7 +15655,7 @@
           <t>8</t>
         </is>
       </c>
-      <c r="B10" s="20" t="inlineStr">
+      <c r="B10" s="38" t="inlineStr">
         <is>
           <t>AAU dorm</t>
         </is>
@@ -15673,7 +15755,7 @@
           <t>9</t>
         </is>
       </c>
-      <c r="B11" s="20" t="inlineStr">
+      <c r="B11" s="38" t="inlineStr">
         <is>
           <t>FOUND Study SF</t>
         </is>
@@ -15777,7 +15859,7 @@
           <t>10</t>
         </is>
       </c>
-      <c r="B12" s="20" t="inlineStr">
+      <c r="B12" s="38" t="inlineStr">
         <is>
           <t>Mosser SRO</t>
         </is>
@@ -15881,7 +15963,7 @@
           <t>11</t>
         </is>
       </c>
-      <c r="B13" s="20" t="inlineStr">
+      <c r="B13" s="38" t="inlineStr">
         <is>
           <t>524 Columbus Residences</t>
         </is>
@@ -15973,7 +16055,7 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B14" s="20" t="inlineStr">
+      <c r="B14" s="38" t="inlineStr">
         <is>
           <t>1055-1069 Pine St</t>
         </is>
@@ -16073,7 +16155,7 @@
           <t>13</t>
         </is>
       </c>
-      <c r="B15" s="20" t="inlineStr">
+      <c r="B15" s="38" t="inlineStr">
         <is>
           <t>Monroe Residence Club</t>
         </is>
@@ -16173,7 +16255,7 @@
           <t>14</t>
         </is>
       </c>
-      <c r="B16" s="20" t="inlineStr">
+      <c r="B16" s="38" t="inlineStr">
         <is>
           <t>Crystal Hotel</t>
         </is>
@@ -16277,7 +16359,7 @@
           <t>15</t>
         </is>
       </c>
-      <c r="B17" s="20" t="inlineStr">
+      <c r="B17" s="38" t="inlineStr">
         <is>
           <t>Sweden House</t>
         </is>
@@ -16377,7 +16459,7 @@
           <t>16</t>
         </is>
       </c>
-      <c r="B18" s="20" t="inlineStr">
+      <c r="B18" s="38" t="inlineStr">
         <is>
           <t>Kenmore Residence Club</t>
         </is>
@@ -16477,7 +16559,7 @@
           <t>17</t>
         </is>
       </c>
-      <c r="B19" s="20" t="inlineStr">
+      <c r="B19" s="38" t="inlineStr">
         <is>
           <t>Villages at Treasure Island</t>
         </is>
@@ -16577,7 +16659,7 @@
           <t>18</t>
         </is>
       </c>
-      <c r="B20" s="20" t="inlineStr">
+      <c r="B20" s="38" t="inlineStr">
         <is>
           <t>CCA surplus dorms</t>
         </is>
@@ -16677,7 +16759,7 @@
           <t>19</t>
         </is>
       </c>
-      <c r="B21" s="20" t="inlineStr">
+      <c r="B21" s="38" t="inlineStr">
         <is>
           <t>1538 Polk St + AAU cluster pairing</t>
         </is>
@@ -16777,7 +16859,7 @@
           <t>20</t>
         </is>
       </c>
-      <c r="B22" s="20" t="inlineStr">
+      <c r="B22" s="38" t="inlineStr">
         <is>
           <t>Parkmerced</t>
         </is>
@@ -16877,7 +16959,7 @@
           <t>21</t>
         </is>
       </c>
-      <c r="B23" s="20" t="inlineStr">
+      <c r="B23" s="38" t="inlineStr">
         <is>
           <t>Foundry Coliving (4 houses)</t>
         </is>
@@ -16977,7 +17059,7 @@
           <t>22</t>
         </is>
       </c>
-      <c r="B24" s="20" t="inlineStr">
+      <c r="B24" s="38" t="inlineStr">
         <is>
           <t>Embassy Hotel</t>
         </is>
@@ -17077,7 +17159,7 @@
           <t>23</t>
         </is>
       </c>
-      <c r="B25" s="20" t="inlineStr">
+      <c r="B25" s="38" t="inlineStr">
         <is>
           <t>Hotel Union Square</t>
         </is>
@@ -17177,7 +17259,7 @@
           <t>24</t>
         </is>
       </c>
-      <c r="B26" s="20" t="inlineStr">
+      <c r="B26" s="38" t="inlineStr">
         <is>
           <t>Motel 6 Civic Center</t>
         </is>
@@ -17281,7 +17363,7 @@
           <t>25</t>
         </is>
       </c>
-      <c r="B27" s="20" t="inlineStr">
+      <c r="B27" s="38" t="inlineStr">
         <is>
           <t>Stanford Court</t>
         </is>
@@ -17381,7 +17463,7 @@
           <t>26</t>
         </is>
       </c>
-      <c r="B28" s="20" t="inlineStr">
+      <c r="B28" s="38" t="inlineStr">
         <is>
           <t>Union Square Plaza Hotel</t>
         </is>
@@ -17481,7 +17563,7 @@
           <t>27</t>
         </is>
       </c>
-      <c r="B29" s="20" t="inlineStr">
+      <c r="B29" s="38" t="inlineStr">
         <is>
           <t>St. Anne's Home</t>
         </is>
@@ -17572,36 +17654,36 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="21" t="str"/>
-      <c r="B30" s="22" t="inlineStr">
+      <c r="A30" s="39" t="str"/>
+      <c r="B30" s="40" t="inlineStr">
         <is>
           <t>--- no phone on file yet (10): find a number, then they join the queue ---</t>
         </is>
       </c>
-      <c r="C30" s="21" t="str"/>
-      <c r="D30" s="21" t="str"/>
-      <c r="E30" s="21" t="str"/>
-      <c r="F30" s="21" t="str"/>
-      <c r="G30" s="21" t="str"/>
-      <c r="H30" s="21" t="str"/>
-      <c r="I30" s="21" t="str"/>
-      <c r="J30" s="21" t="str"/>
-      <c r="K30" s="21" t="str"/>
-      <c r="L30" s="21" t="str"/>
-      <c r="M30" s="21" t="str"/>
-      <c r="N30" s="21" t="str"/>
-      <c r="O30" s="21" t="str"/>
-      <c r="P30" s="21" t="str"/>
-      <c r="Q30" s="21" t="str"/>
-      <c r="R30" s="21" t="str"/>
-      <c r="S30" s="21" t="str"/>
-      <c r="T30" s="21" t="str"/>
-      <c r="U30" s="21" t="str"/>
-      <c r="V30" s="21" t="str"/>
+      <c r="C30" s="39" t="str"/>
+      <c r="D30" s="39" t="str"/>
+      <c r="E30" s="39" t="str"/>
+      <c r="F30" s="39" t="str"/>
+      <c r="G30" s="39" t="str"/>
+      <c r="H30" s="39" t="str"/>
+      <c r="I30" s="39" t="str"/>
+      <c r="J30" s="39" t="str"/>
+      <c r="K30" s="39" t="str"/>
+      <c r="L30" s="39" t="str"/>
+      <c r="M30" s="39" t="str"/>
+      <c r="N30" s="39" t="str"/>
+      <c r="O30" s="39" t="str"/>
+      <c r="P30" s="39" t="str"/>
+      <c r="Q30" s="39" t="str"/>
+      <c r="R30" s="39" t="str"/>
+      <c r="S30" s="39" t="str"/>
+      <c r="T30" s="39" t="str"/>
+      <c r="U30" s="39" t="str"/>
+      <c r="V30" s="39" t="str"/>
     </row>
     <row r="31">
       <c r="A31" s="7" t="str"/>
-      <c r="B31" s="20" t="inlineStr">
+      <c r="B31" s="38" t="inlineStr">
         <is>
           <t>Panoramic Residences</t>
         </is>
@@ -17685,7 +17767,7 @@
     </row>
     <row r="32">
       <c r="A32" s="7" t="str"/>
-      <c r="B32" s="20" t="inlineStr">
+      <c r="B32" s="38" t="inlineStr">
         <is>
           <t>City Gardens Apartments</t>
         </is>
@@ -17765,7 +17847,7 @@
     </row>
     <row r="33">
       <c r="A33" s="7" t="str"/>
-      <c r="B33" s="20" t="inlineStr">
+      <c r="B33" s="38" t="inlineStr">
         <is>
           <t>SOMA Residences</t>
         </is>
@@ -17845,7 +17927,7 @@
     </row>
     <row r="34">
       <c r="A34" s="7" t="str"/>
-      <c r="B34" s="20" t="inlineStr">
+      <c r="B34" s="38" t="inlineStr">
         <is>
           <t>149-161 Hyde St</t>
         </is>
@@ -17945,7 +18027,7 @@
     </row>
     <row r="35">
       <c r="A35" s="7" t="str"/>
-      <c r="B35" s="20" t="inlineStr">
+      <c r="B35" s="38" t="inlineStr">
         <is>
           <t>TL Residences</t>
         </is>
@@ -18029,7 +18111,7 @@
     </row>
     <row r="36">
       <c r="A36" s="7" t="str"/>
-      <c r="B36" s="20" t="inlineStr">
+      <c r="B36" s="38" t="inlineStr">
         <is>
           <t>20 Mission SF (20mish)</t>
         </is>
@@ -18133,7 +18215,7 @@
     </row>
     <row r="37">
       <c r="A37" s="7" t="str"/>
-      <c r="B37" s="20" t="inlineStr">
+      <c r="B37" s="38" t="inlineStr">
         <is>
           <t>20mish</t>
         </is>
@@ -18229,7 +18311,7 @@
     </row>
     <row r="38">
       <c r="A38" s="7" t="str"/>
-      <c r="B38" s="20" t="inlineStr">
+      <c r="B38" s="38" t="inlineStr">
         <is>
           <t>Hotel Fiona</t>
         </is>
@@ -18309,7 +18391,7 @@
     </row>
     <row r="39">
       <c r="A39" s="7" t="str"/>
-      <c r="B39" s="20" t="inlineStr">
+      <c r="B39" s="38" t="inlineStr">
         <is>
           <t>Hotel Whitcomb floors</t>
         </is>
@@ -18409,7 +18491,7 @@
     </row>
     <row r="40">
       <c r="A40" s="7" t="str"/>
-      <c r="B40" s="20" t="inlineStr">
+      <c r="B40" s="38" t="inlineStr">
         <is>
           <t>Salvation Army McFee Center</t>
         </is>
@@ -18541,7 +18623,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="56" customHeight="1">
-      <c r="A1" s="19" t="inlineStr">
+      <c r="A1" s="37" t="inlineStr">
         <is>
           <t>Femme / safe house: about 10 to 12 women, kitchen required, 3 to 6 months. 2550 Van Ness (Minerva) is the live option; these are backups in calling order. Safety column matters double here. Calls made with Granola get logged onto the row by Claude.</t>
         </is>
@@ -18665,7 +18747,7 @@
           <t>1</t>
         </is>
       </c>
-      <c r="B3" s="20" t="inlineStr">
+      <c r="B3" s="38" t="inlineStr">
         <is>
           <t>Hive Coliving (was Tribe)</t>
         </is>
@@ -18769,7 +18851,7 @@
           <t>2</t>
         </is>
       </c>
-      <c r="B4" s="20" t="inlineStr">
+      <c r="B4" s="38" t="inlineStr">
         <is>
           <t>AAU dorm</t>
         </is>
@@ -18869,7 +18951,7 @@
           <t>3</t>
         </is>
       </c>
-      <c r="B5" s="20" t="inlineStr">
+      <c r="B5" s="38" t="inlineStr">
         <is>
           <t>FOUND Study SF</t>
         </is>
@@ -18973,7 +19055,7 @@
           <t>4</t>
         </is>
       </c>
-      <c r="B6" s="20" t="inlineStr">
+      <c r="B6" s="38" t="inlineStr">
         <is>
           <t>The Bartlett Residences</t>
         </is>
@@ -19065,7 +19147,7 @@
           <t>5</t>
         </is>
       </c>
-      <c r="B7" s="20" t="inlineStr">
+      <c r="B7" s="38" t="inlineStr">
         <is>
           <t>The Herbert Residences</t>
         </is>
@@ -19157,7 +19239,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="B8" s="20" t="inlineStr">
+      <c r="B8" s="38" t="inlineStr">
         <is>
           <t>Boston Hotel (SRO)</t>
         </is>
@@ -19261,7 +19343,7 @@
           <t>7</t>
         </is>
       </c>
-      <c r="B9" s="20" t="inlineStr">
+      <c r="B9" s="38" t="inlineStr">
         <is>
           <t>Monroe Residence Club</t>
         </is>
@@ -19361,7 +19443,7 @@
           <t>8</t>
         </is>
       </c>
-      <c r="B10" s="20" t="inlineStr">
+      <c r="B10" s="38" t="inlineStr">
         <is>
           <t>Kenmore Residence Club</t>
         </is>
@@ -19461,7 +19543,7 @@
           <t>9</t>
         </is>
       </c>
-      <c r="B11" s="20" t="inlineStr">
+      <c r="B11" s="38" t="inlineStr">
         <is>
           <t>Hotel Epik Residences</t>
         </is>
@@ -19553,7 +19635,7 @@
           <t>10</t>
         </is>
       </c>
-      <c r="B12" s="20" t="inlineStr">
+      <c r="B12" s="38" t="inlineStr">
         <is>
           <t>Lovely North Beach / Chinatown Hotel</t>
         </is>
@@ -19645,7 +19727,7 @@
           <t>11</t>
         </is>
       </c>
-      <c r="B13" s="20" t="inlineStr">
+      <c r="B13" s="38" t="inlineStr">
         <is>
           <t>2436 Mission Residences</t>
         </is>
@@ -19737,7 +19819,7 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B14" s="20" t="inlineStr">
+      <c r="B14" s="38" t="inlineStr">
         <is>
           <t>Blue Hotel</t>
         </is>
@@ -19837,7 +19919,7 @@
           <t>13</t>
         </is>
       </c>
-      <c r="B15" s="20" t="inlineStr">
+      <c r="B15" s="38" t="inlineStr">
         <is>
           <t>The Perramont</t>
         </is>
@@ -19929,7 +20011,7 @@
           <t>14</t>
         </is>
       </c>
-      <c r="B16" s="20" t="inlineStr">
+      <c r="B16" s="38" t="inlineStr">
         <is>
           <t>Presidio Residences</t>
         </is>
@@ -20024,36 +20106,36 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="21" t="str"/>
-      <c r="B17" s="22" t="inlineStr">
+      <c r="A17" s="39" t="str"/>
+      <c r="B17" s="40" t="inlineStr">
         <is>
           <t>--- no phone on file yet (2): find a number, then they join the queue ---</t>
         </is>
       </c>
-      <c r="C17" s="21" t="str"/>
-      <c r="D17" s="21" t="str"/>
-      <c r="E17" s="21" t="str"/>
-      <c r="F17" s="21" t="str"/>
-      <c r="G17" s="21" t="str"/>
-      <c r="H17" s="21" t="str"/>
-      <c r="I17" s="21" t="str"/>
-      <c r="J17" s="21" t="str"/>
-      <c r="K17" s="21" t="str"/>
-      <c r="L17" s="21" t="str"/>
-      <c r="M17" s="21" t="str"/>
-      <c r="N17" s="21" t="str"/>
-      <c r="O17" s="21" t="str"/>
-      <c r="P17" s="21" t="str"/>
-      <c r="Q17" s="21" t="str"/>
-      <c r="R17" s="21" t="str"/>
-      <c r="S17" s="21" t="str"/>
-      <c r="T17" s="21" t="str"/>
-      <c r="U17" s="21" t="str"/>
-      <c r="V17" s="21" t="str"/>
+      <c r="C17" s="39" t="str"/>
+      <c r="D17" s="39" t="str"/>
+      <c r="E17" s="39" t="str"/>
+      <c r="F17" s="39" t="str"/>
+      <c r="G17" s="39" t="str"/>
+      <c r="H17" s="39" t="str"/>
+      <c r="I17" s="39" t="str"/>
+      <c r="J17" s="39" t="str"/>
+      <c r="K17" s="39" t="str"/>
+      <c r="L17" s="39" t="str"/>
+      <c r="M17" s="39" t="str"/>
+      <c r="N17" s="39" t="str"/>
+      <c r="O17" s="39" t="str"/>
+      <c r="P17" s="39" t="str"/>
+      <c r="Q17" s="39" t="str"/>
+      <c r="R17" s="39" t="str"/>
+      <c r="S17" s="39" t="str"/>
+      <c r="T17" s="39" t="str"/>
+      <c r="U17" s="39" t="str"/>
+      <c r="V17" s="39" t="str"/>
     </row>
     <row r="18">
       <c r="A18" s="7" t="str"/>
-      <c r="B18" s="20" t="inlineStr">
+      <c r="B18" s="38" t="inlineStr">
         <is>
           <t>20mish</t>
         </is>
@@ -20149,7 +20231,7 @@
     </row>
     <row r="19">
       <c r="A19" s="7" t="str"/>
-      <c r="B19" s="20" t="inlineStr">
+      <c r="B19" s="38" t="inlineStr">
         <is>
           <t>The Red Victorian</t>
         </is>
@@ -20269,7 +20351,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="56" customHeight="1">
-      <c r="A1" s="19" t="inlineStr">
+      <c r="A1" s="37" t="inlineStr">
         <is>
           <t>Alum house and spillover: operating co-living, hostels and SROs under ~35 beds where one person can just book in. Call in order to confirm rates and holds; Granola notes get logged onto the row. Hive: toured by Elliot, great community reviews, no block available, actively looking for female residents.</t>
         </is>
@@ -20393,7 +20475,7 @@
           <t>1</t>
         </is>
       </c>
-      <c r="B3" s="20" t="inlineStr">
+      <c r="B3" s="38" t="inlineStr">
         <is>
           <t>221 7th Street Residences</t>
         </is>
@@ -20497,7 +20579,7 @@
           <t>2</t>
         </is>
       </c>
-      <c r="B4" s="20" t="inlineStr">
+      <c r="B4" s="38" t="inlineStr">
         <is>
           <t>251 9th Street Residences</t>
         </is>
@@ -20589,7 +20671,7 @@
           <t>3</t>
         </is>
       </c>
-      <c r="B5" s="20" t="inlineStr">
+      <c r="B5" s="38" t="inlineStr">
         <is>
           <t>European Hostel</t>
         </is>
@@ -20697,7 +20779,7 @@
           <t>4</t>
         </is>
       </c>
-      <c r="B6" s="20" t="inlineStr">
+      <c r="B6" s="38" t="inlineStr">
         <is>
           <t>UrbaNests 1080 Folsom Residences</t>
         </is>
@@ -20793,7 +20875,7 @@
           <t>5</t>
         </is>
       </c>
-      <c r="B7" s="20" t="inlineStr">
+      <c r="B7" s="38" t="inlineStr">
         <is>
           <t>The Bartlett Residences</t>
         </is>
@@ -20885,7 +20967,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="B8" s="20" t="inlineStr">
+      <c r="B8" s="38" t="inlineStr">
         <is>
           <t>The Herbert Residences</t>
         </is>
@@ -20977,7 +21059,7 @@
           <t>7</t>
         </is>
       </c>
-      <c r="B9" s="20" t="inlineStr">
+      <c r="B9" s="38" t="inlineStr">
         <is>
           <t>1214 Polk Street Residences</t>
         </is>
@@ -21069,7 +21151,7 @@
           <t>8</t>
         </is>
       </c>
-      <c r="B10" s="20" t="inlineStr">
+      <c r="B10" s="38" t="inlineStr">
         <is>
           <t>371 Columbus Residences</t>
         </is>
@@ -21161,7 +21243,7 @@
           <t>9</t>
         </is>
       </c>
-      <c r="B11" s="20" t="inlineStr">
+      <c r="B11" s="38" t="inlineStr">
         <is>
           <t>Hotel Epik Residences</t>
         </is>
@@ -21253,7 +21335,7 @@
           <t>10</t>
         </is>
       </c>
-      <c r="B12" s="20" t="inlineStr">
+      <c r="B12" s="38" t="inlineStr">
         <is>
           <t>556 Green St Residences</t>
         </is>
@@ -21345,7 +21427,7 @@
           <t>11</t>
         </is>
       </c>
-      <c r="B13" s="20" t="inlineStr">
+      <c r="B13" s="38" t="inlineStr">
         <is>
           <t>2436 Mission Residences</t>
         </is>
@@ -21437,7 +21519,7 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B14" s="20" t="inlineStr">
+      <c r="B14" s="38" t="inlineStr">
         <is>
           <t>Hive Coliving (was Tribe)</t>
         </is>
@@ -21545,7 +21627,7 @@
           <t>13</t>
         </is>
       </c>
-      <c r="B15" s="20" t="inlineStr">
+      <c r="B15" s="38" t="inlineStr">
         <is>
           <t>Monroe Residence Club</t>
         </is>
@@ -21637,7 +21719,7 @@
           <t>14</t>
         </is>
       </c>
-      <c r="B16" s="20" t="inlineStr">
+      <c r="B16" s="38" t="inlineStr">
         <is>
           <t>Kenmore Residence Hotel</t>
         </is>
@@ -21729,7 +21811,7 @@
           <t>15</t>
         </is>
       </c>
-      <c r="B17" s="20" t="inlineStr">
+      <c r="B17" s="38" t="inlineStr">
         <is>
           <t>Hive Coliving (bunks)</t>
         </is>
@@ -21821,7 +21903,7 @@
           <t>16</t>
         </is>
       </c>
-      <c r="B18" s="20" t="inlineStr">
+      <c r="B18" s="38" t="inlineStr">
         <is>
           <t>The Perramont</t>
         </is>
@@ -21913,7 +21995,7 @@
           <t>17</t>
         </is>
       </c>
-      <c r="B19" s="20" t="inlineStr">
+      <c r="B19" s="38" t="inlineStr">
         <is>
           <t>Foundry Coliving</t>
         </is>
@@ -22004,36 +22086,36 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="21" t="str"/>
-      <c r="B20" s="22" t="inlineStr">
+      <c r="A20" s="39" t="str"/>
+      <c r="B20" s="40" t="inlineStr">
         <is>
           <t>--- no phone on file yet (21): find a number, then they join the queue ---</t>
         </is>
       </c>
-      <c r="C20" s="21" t="str"/>
-      <c r="D20" s="21" t="str"/>
-      <c r="E20" s="21" t="str"/>
-      <c r="F20" s="21" t="str"/>
-      <c r="G20" s="21" t="str"/>
-      <c r="H20" s="21" t="str"/>
-      <c r="I20" s="21" t="str"/>
-      <c r="J20" s="21" t="str"/>
-      <c r="K20" s="21" t="str"/>
-      <c r="L20" s="21" t="str"/>
-      <c r="M20" s="21" t="str"/>
-      <c r="N20" s="21" t="str"/>
-      <c r="O20" s="21" t="str"/>
-      <c r="P20" s="21" t="str"/>
-      <c r="Q20" s="21" t="str"/>
-      <c r="R20" s="21" t="str"/>
-      <c r="S20" s="21" t="str"/>
-      <c r="T20" s="21" t="str"/>
-      <c r="U20" s="21" t="str"/>
-      <c r="V20" s="21" t="str"/>
+      <c r="C20" s="39" t="str"/>
+      <c r="D20" s="39" t="str"/>
+      <c r="E20" s="39" t="str"/>
+      <c r="F20" s="39" t="str"/>
+      <c r="G20" s="39" t="str"/>
+      <c r="H20" s="39" t="str"/>
+      <c r="I20" s="39" t="str"/>
+      <c r="J20" s="39" t="str"/>
+      <c r="K20" s="39" t="str"/>
+      <c r="L20" s="39" t="str"/>
+      <c r="M20" s="39" t="str"/>
+      <c r="N20" s="39" t="str"/>
+      <c r="O20" s="39" t="str"/>
+      <c r="P20" s="39" t="str"/>
+      <c r="Q20" s="39" t="str"/>
+      <c r="R20" s="39" t="str"/>
+      <c r="S20" s="39" t="str"/>
+      <c r="T20" s="39" t="str"/>
+      <c r="U20" s="39" t="str"/>
+      <c r="V20" s="39" t="str"/>
     </row>
     <row r="21">
       <c r="A21" s="7" t="str"/>
-      <c r="B21" s="20" t="inlineStr">
+      <c r="B21" s="38" t="inlineStr">
         <is>
           <t>HI San Francisco Downtown</t>
         </is>
@@ -22117,7 +22199,7 @@
     </row>
     <row r="22">
       <c r="A22" s="7" t="str"/>
-      <c r="B22" s="20" t="inlineStr">
+      <c r="B22" s="38" t="inlineStr">
         <is>
           <t>Amsterdam Hostel</t>
         </is>
@@ -22209,7 +22291,7 @@
     </row>
     <row r="23">
       <c r="A23" s="7" t="str"/>
-      <c r="B23" s="20" t="inlineStr">
+      <c r="B23" s="38" t="inlineStr">
         <is>
           <t>Orange Village Hostel</t>
         </is>
@@ -22297,7 +22379,7 @@
     </row>
     <row r="24">
       <c r="A24" s="7" t="str"/>
-      <c r="B24" s="20" t="inlineStr">
+      <c r="B24" s="38" t="inlineStr">
         <is>
           <t>Adelaide Hostel</t>
         </is>
@@ -22373,7 +22455,7 @@
     </row>
     <row r="25">
       <c r="A25" s="7" t="str"/>
-      <c r="B25" s="20" t="inlineStr">
+      <c r="B25" s="38" t="inlineStr">
         <is>
           <t>ITH Pacific Tradewinds</t>
         </is>
@@ -22449,7 +22531,7 @@
     </row>
     <row r="26">
       <c r="A26" s="7" t="str"/>
-      <c r="B26" s="20" t="inlineStr">
+      <c r="B26" s="38" t="inlineStr">
         <is>
           <t>Bposhtels SF Union Square</t>
         </is>
@@ -22529,7 +22611,7 @@
     </row>
     <row r="27">
       <c r="A27" s="7" t="str"/>
-      <c r="B27" s="20" t="inlineStr">
+      <c r="B27" s="38" t="inlineStr">
         <is>
           <t>Green Tortoise Hostel</t>
         </is>
@@ -22605,7 +22687,7 @@
     </row>
     <row r="28">
       <c r="A28" s="7" t="str"/>
-      <c r="B28" s="20" t="inlineStr">
+      <c r="B28" s="38" t="inlineStr">
         <is>
           <t>Samesun San Francisco</t>
         </is>
@@ -22685,7 +22767,7 @@
     </row>
     <row r="29">
       <c r="A29" s="7" t="str"/>
-      <c r="B29" s="20" t="inlineStr">
+      <c r="B29" s="38" t="inlineStr">
         <is>
           <t>The Annex at Hayes Valley</t>
         </is>
@@ -22761,7 +22843,7 @@
     </row>
     <row r="30">
       <c r="A30" s="7" t="str"/>
-      <c r="B30" s="20" t="inlineStr">
+      <c r="B30" s="38" t="inlineStr">
         <is>
           <t>The 6th Collective Coliving</t>
         </is>
@@ -22845,7 +22927,7 @@
     </row>
     <row r="31">
       <c r="A31" s="7" t="str"/>
-      <c r="B31" s="20" t="inlineStr">
+      <c r="B31" s="38" t="inlineStr">
         <is>
           <t>Chapter San Francisco</t>
         </is>
@@ -22921,7 +23003,7 @@
     </row>
     <row r="32">
       <c r="A32" s="7" t="str"/>
-      <c r="B32" s="20" t="inlineStr">
+      <c r="B32" s="38" t="inlineStr">
         <is>
           <t>Harcourt Hotel (residence)</t>
         </is>
@@ -23001,7 +23083,7 @@
     </row>
     <row r="33">
       <c r="A33" s="7" t="str"/>
-      <c r="B33" s="20" t="inlineStr">
+      <c r="B33" s="38" t="inlineStr">
         <is>
           <t>Vybe Living (operator)</t>
         </is>
@@ -23077,7 +23159,7 @@
     </row>
     <row r="34">
       <c r="A34" s="7" t="str"/>
-      <c r="B34" s="20" t="inlineStr">
+      <c r="B34" s="38" t="inlineStr">
         <is>
           <t>HI Fisherman's Wharf Hostel</t>
         </is>
@@ -23157,7 +23239,7 @@
     </row>
     <row r="35">
       <c r="A35" s="7" t="str"/>
-      <c r="B35" s="20" t="inlineStr">
+      <c r="B35" s="38" t="inlineStr">
         <is>
           <t>Blok Living Lower Haight</t>
         </is>
@@ -23233,7 +23315,7 @@
     </row>
     <row r="36">
       <c r="A36" s="7" t="str"/>
-      <c r="B36" s="20" t="inlineStr">
+      <c r="B36" s="38" t="inlineStr">
         <is>
           <t>Furnished Quarters SF</t>
         </is>
@@ -23309,7 +23391,7 @@
     </row>
     <row r="37">
       <c r="A37" s="7" t="str"/>
-      <c r="B37" s="20" t="inlineStr">
+      <c r="B37" s="38" t="inlineStr">
         <is>
           <t>PodShare SF Marina</t>
         </is>
@@ -23385,7 +23467,7 @@
     </row>
     <row r="38">
       <c r="A38" s="7" t="str"/>
-      <c r="B38" s="20" t="inlineStr">
+      <c r="B38" s="38" t="inlineStr">
         <is>
           <t>Mission Control</t>
         </is>
@@ -23461,7 +23543,7 @@
     </row>
     <row r="39">
       <c r="A39" s="7" t="str"/>
-      <c r="B39" s="20" t="inlineStr">
+      <c r="B39" s="38" t="inlineStr">
         <is>
           <t>The Red Victorian</t>
         </is>
@@ -23541,7 +23623,7 @@
     </row>
     <row r="40">
       <c r="A40" s="7" t="str"/>
-      <c r="B40" s="20" t="inlineStr">
+      <c r="B40" s="38" t="inlineStr">
         <is>
           <t>Mission Dolores Manor</t>
         </is>
@@ -23617,7 +23699,7 @@
     </row>
     <row r="41">
       <c r="A41" s="7" t="str"/>
-      <c r="B41" s="20" t="inlineStr">
+      <c r="B41" s="38" t="inlineStr">
         <is>
           <t>908 Coliving</t>
         </is>
@@ -23733,22 +23815,22 @@
       </c>
     </row>
     <row r="2" ht="150" customHeight="1">
-      <c r="A2" s="23" t="inlineStr">
+      <c r="A2" s="41" t="inlineStr">
         <is>
           <t>original-team-template</t>
         </is>
       </c>
-      <c r="B2" s="23" t="inlineStr">
+      <c r="B2" s="41" t="inlineStr">
         <is>
           <t>Reference - what Alex/Giulia already send (10-15 rooms, 3-6 months)</t>
         </is>
       </c>
-      <c r="C2" s="23" t="inlineStr">
+      <c r="C2" s="41" t="inlineStr">
         <is>
           <t>Group housing inquiry - Biopunk/Haus Fund</t>
         </is>
       </c>
-      <c r="D2" s="23" t="inlineStr">
+      <c r="D2" s="41" t="inlineStr">
         <is>
           <t>To whom it may concern,
 Hi. My name is [NAME], and I'm scouting properties with my colleague [COLLEAGUE] that could be a good fit for our organisation Biopunk/Haus Fund. We are a fast-growing startup community based in SF, running a network of founder houses focused on biotech and entrepreneurship. Flagship house: https://biopunk.house · Program info: https://haus.fund
@@ -23761,44 +23843,44 @@
       </c>
     </row>
     <row r="3" ht="150" customHeight="1">
-      <c r="A3" s="23" t="inlineStr">
+      <c r="A3" s="41" t="inlineStr">
         <is>
           <t>call-script-60s</t>
         </is>
       </c>
-      <c r="B3" s="23" t="inlineStr">
+      <c r="B3" s="41" t="inlineStr">
         <is>
           <t>Phone follow-up when email gets no reply in 10 days</t>
         </is>
       </c>
-      <c r="C3" s="23" t="inlineStr">
+      <c r="C3" s="41" t="inlineStr">
         <is>
           <t xml:space="preserve"> - </t>
         </is>
       </c>
-      <c r="D3" s="23" t="inlineStr">
+      <c r="D3" s="41" t="inlineStr">
         <is>
           <t>"Hi, this is {{sender_name}} from Biopunk, an accelerator in SF. We house 40-50 founders each program and {{name}} is on our list. Three quick questions: how many rooms could you offer from Sept 15 for 30-plus nights? What's the monthly rate for a group? And is there kitchen access? … Great - can I send you a one-paragraph email with our details so you have it in writing? What's the best address?" (Log the answers in the Outreach log.)</t>
         </is>
       </c>
     </row>
     <row r="4" ht="150" customHeight="1">
-      <c r="A4" s="23" t="inlineStr">
+      <c r="A4" s="41" t="inlineStr">
         <is>
           <t>co-living-block</t>
         </is>
       </c>
-      <c r="B4" s="23" t="inlineStr">
+      <c r="B4" s="41" t="inlineStr">
         <is>
           <t>Operators: FOUND Study, UpMarket/221 7th, Urbanests, Hive, Foundry, 20mish, Brownstone, hostels</t>
         </is>
       </c>
-      <c r="C4" s="23" t="inlineStr">
+      <c r="C4" s="41" t="inlineStr">
         <is>
           <t>Block booking - 40-50 beds, 30+ nights, recurring</t>
         </is>
       </c>
-      <c r="D4" s="23" t="inlineStr">
+      <c r="D4" s="41" t="inlineStr">
         <is>
           <t>Hi {{contact_name}},
 Biopunk (biopunk.house) houses 40-50 founders in SF every program cycle and we'd like to make {{name}} one of our standing options. We're looking for a block of beds from Sept 15 - mix of private and shared is fine - with 30+ day stays, kitchen access, and a group rate.
@@ -23811,22 +23893,22 @@
       </c>
     </row>
     <row r="5" ht="150" customHeight="1">
-      <c r="A5" s="23" t="inlineStr">
+      <c r="A5" s="41" t="inlineStr">
         <is>
           <t>dorm-institution</t>
         </is>
       </c>
-      <c r="B5" s="23" t="inlineStr">
+      <c r="B5" s="41" t="inlineStr">
         <is>
           <t>Academy of Art, CCA, Holy Names, NDNU - never mention the residency</t>
         </is>
       </c>
-      <c r="C5" s="23" t="inlineStr">
+      <c r="C5" s="41" t="inlineStr">
         <is>
           <t>Residence hall lease for an accelerator cohort - 40-50 beds</t>
         </is>
       </c>
-      <c r="D5" s="23" t="inlineStr">
+      <c r="D5" s="41" t="inlineStr">
         <is>
           <t>Hi {{contact_name}},
 I'm writing on behalf of Biopunk, a large San Francisco accelerator for biotech founders (biopunk.house). Each cohort brings 40-50 residents to the city for a program term, and we're looking for purpose-built student or residence-hall housing rather than hotels.
@@ -23839,22 +23921,22 @@
       </c>
     </row>
     <row r="6" ht="150" customHeight="1">
-      <c r="A6" s="23" t="inlineStr">
+      <c r="A6" s="41" t="inlineStr">
         <is>
           <t>femme-house</t>
         </is>
       </c>
-      <c r="B6" s="23" t="inlineStr">
+      <c r="B6" s="41" t="inlineStr">
         <is>
           <t>Femhaus - ~10-12 women, kitchen required, 3-6 months</t>
         </is>
       </c>
-      <c r="C6" s="23" t="inlineStr">
+      <c r="C6" s="41" t="inlineStr">
         <is>
           <t>Small group housing - 10-12 residents, 3-6 months, kitchen required</t>
         </is>
       </c>
-      <c r="D6" s="23" t="inlineStr">
+      <c r="D6" s="41" t="inlineStr">
         <is>
           <t>Hi {{contact_name}},
 Biopunk runs a women-founder residence (Femhaus) within our SF accelerator and we're placing 10-12 residents from Sept 15 for 3-6 months, ideally in one building or one floor. A full kitchen on site is a requirement, private rooms preferred, shared is possible.
@@ -23866,22 +23948,22 @@
       </c>
     </row>
     <row r="7" ht="150" customHeight="1">
-      <c r="A7" s="23" t="inlineStr">
+      <c r="A7" s="41" t="inlineStr">
         <is>
           <t>receiver-or-lender</t>
         </is>
       </c>
-      <c r="B7" s="23" t="inlineStr">
+      <c r="B7" s="41" t="inlineStr">
         <is>
           <t>Receivers, special servicers, lender-REO (Moxy, Stanford Court, Whitcomb, Ora, Moran)</t>
         </is>
       </c>
-      <c r="C7" s="23" t="inlineStr">
+      <c r="C7" s="41" t="inlineStr">
         <is>
           <t>Guaranteed master lease on {{name}} - income while you decide</t>
         </is>
       </c>
-      <c r="D7" s="23" t="inlineStr">
+      <c r="D7" s="41" t="inlineStr">
         <is>
           <t>Hi {{contact_name}},
 I represent Biopunk, an SF accelerator with 40-50 residents per cohort. I understand {{name}} ({{address}}) is currently generating little or no income pending resolution. We'd like to propose a guaranteed master lease of {{rooms}} rooms, 2-5 years with renewal, at around {{price_ask}}/room/month, with a purchase option at a pre-agreed price - converting a dark asset to income while you run your process.
@@ -23893,22 +23975,22 @@
       </c>
     </row>
     <row r="8" ht="150" customHeight="1">
-      <c r="A8" s="23" t="inlineStr">
+      <c r="A8" s="41" t="inlineStr">
         <is>
           <t>sro-master-lease</t>
         </is>
       </c>
-      <c r="B8" s="23" t="inlineStr">
+      <c r="B8" s="41" t="inlineStr">
         <is>
           <t>SRO / residential hotels (Crystal, Mosser, Boston, Harcourt, Mission Hotel Apts)</t>
         </is>
       </c>
-      <c r="C8" s="23" t="inlineStr">
+      <c r="C8" s="41" t="inlineStr">
         <is>
           <t>Whole-building residential master lease - 45 rooms, credit tenant</t>
         </is>
       </c>
-      <c r="D8" s="23" t="inlineStr">
+      <c r="D8" s="41" t="inlineStr">
         <is>
           <t>Hi {{contact_name}},
 I represent Biopunk, a San Francisco accelerator that houses 40-50 founders year-round (biopunk.house · haus.fund). We're looking for a 5-10 year residential master lease of a single building in the 35-60 room range and {{name}} at {{address}} fits.
@@ -23921,22 +24003,22 @@
       </c>
     </row>
     <row r="9" ht="150" customHeight="1">
-      <c r="A9" s="23" t="inlineStr">
+      <c r="A9" s="41" t="inlineStr">
         <is>
           <t>weekly-availability-check</t>
         </is>
       </c>
-      <c r="B9" s="23" t="inlineStr">
+      <c r="B9" s="41" t="inlineStr">
         <is>
           <t>The automated weekly email (AI-assisted inbox) to every operator on Inventory</t>
         </is>
       </c>
-      <c r="C9" s="23" t="inlineStr">
+      <c r="C9" s="41" t="inlineStr">
         <is>
           <t>Quick availability check - Biopunk housing ({{month}})</t>
         </is>
       </c>
-      <c r="D9" s="23" t="inlineStr">
+      <c r="D9" s="41" t="inlineStr">
         <is>
           <t>Hi {{contact_name}},
 Quick check for our founders' housing list - three questions:
@@ -23982,7 +24064,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="56" customHeight="1">
-      <c r="A1" s="19" t="inlineStr">
+      <c r="A1" s="37" t="inlineStr">
         <is>
           <t>Rows with status=confirmed, flat columns, ready to import into the Airtable CRM (Google Sheets is for drafting; Airtable is where set-in-stone deals live). Mark a row confirmed and re-run push-to-sheet.</t>
         </is>

</xml_diff>